<commit_message>
Correct canopy leaf areas and refresh analysis outputs
Correct July black-gum tissue and height metadata, share areas across paired foliage closures, and use within-species means for unmatched leaf samples. Centralize area assignments and add metadata consistency checks. Refresh fluxes, scaling results, figures and uncertainty comparisons; document chamber construction with field photographs and strengthen private-file exclusions.
</commit_message>
<xml_diff>
--- a/data processing/goFlux_reprocessing/results/CH4_best_all.xlsx
+++ b/data processing/goFlux_reprocessing/results/CH4_best_all.xlsx
@@ -1445,7 +1445,7 @@
         <v>52</v>
       </c>
       <c r="B5" t="n">
-        <v>-0.00247728792264067</v>
+        <v>-0.00370933885356478</v>
       </c>
       <c r="C5" t="n">
         <v>1966.79506874272</v>
@@ -1466,10 +1466,10 @@
         <v>1333.75046647897</v>
       </c>
       <c r="I5" t="n">
-        <v>0.00228241134129574</v>
+        <v>0.00341754081977201</v>
       </c>
       <c r="J5" t="n">
-        <v>-92.1334706570077</v>
+        <v>-92.133422010978</v>
       </c>
       <c r="K5" t="n">
         <v>0.000714570624363642</v>
@@ -1478,7 +1478,7 @@
         <v>0.278806173790103</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.00262265685640335</v>
+        <v>-0.00392700537071811</v>
       </c>
       <c r="N5" t="n">
         <v>1966.80280348799</v>
@@ -1499,10 +1499,10 @@
         <v>1335.8161372716</v>
       </c>
       <c r="T5" t="n">
-        <v>0.00945398798865747</v>
+        <v>0.0141558137555216</v>
       </c>
       <c r="U5" t="n">
-        <v>-360.473691614481</v>
+        <v>-360.473501286121</v>
       </c>
       <c r="V5" t="n">
         <v>0.000714704680034983</v>
@@ -1517,13 +1517,13 @@
         <v>1966.07</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.0213807284363752</v>
+        <v>0.0320141901882866</v>
       </c>
       <c r="AA5" t="n">
         <v>7.07037944035506</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.749948527791428</v>
+        <v>1.12292688584425</v>
       </c>
       <c r="AC5" t="n">
         <v>250</v>
@@ -1544,7 +1544,7 @@
         <v>54</v>
       </c>
       <c r="AI5" t="n">
-        <v>-0.00262265685640335</v>
+        <v>-0.00392700537071811</v>
       </c>
       <c r="AJ5" t="s">
         <v>49</v>
@@ -1568,7 +1568,7 @@
         <v>0.5</v>
       </c>
       <c r="AQ5" t="n">
-        <v>0.021</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="6">
@@ -1576,7 +1576,7 @@
         <v>56</v>
       </c>
       <c r="B6" t="n">
-        <v>0.00310787992128603</v>
+        <v>0.00398796026045624</v>
       </c>
       <c r="C6" t="n">
         <v>1964.27684003335</v>
@@ -1597,10 +1597,10 @@
         <v>875.495415275172</v>
       </c>
       <c r="I6" t="n">
-        <v>0.00294410482542063</v>
+        <v>0.00377780837102057</v>
       </c>
       <c r="J6" t="n">
-        <v>94.7303274253392</v>
+        <v>94.7303414349563</v>
       </c>
       <c r="K6" t="n">
         <v>0.000638417369216882</v>
@@ -1609,7 +1609,7 @@
         <v>0.292569034510092</v>
       </c>
       <c r="M6" t="n">
-        <v>0.00328454730842572</v>
+        <v>0.00421465580117076</v>
       </c>
       <c r="N6" t="n">
         <v>1964.26911984858</v>
@@ -1630,10 +1630,10 @@
         <v>877.580106611765</v>
       </c>
       <c r="T6" t="n">
-        <v>0.0121933355616092</v>
+        <v>0.0156462109492753</v>
       </c>
       <c r="U6" t="n">
-        <v>371.233366934009</v>
+        <v>371.233421835516</v>
       </c>
       <c r="V6" t="n">
         <v>0.000680147925572583</v>
@@ -1648,13 +1648,13 @@
         <v>1965.13</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.0295436144609756</v>
+        <v>0.0379096887282113</v>
       </c>
       <c r="AA6" t="n">
         <v>7.07037944035506</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.747952360000791</v>
+        <v>0.959755320007132</v>
       </c>
       <c r="AC6" t="n">
         <v>180</v>
@@ -1675,7 +1675,7 @@
         <v>54</v>
       </c>
       <c r="AI6" t="n">
-        <v>0.00328454730842572</v>
+        <v>0.00421465580117076</v>
       </c>
       <c r="AJ6" t="s">
         <v>49</v>
@@ -1699,7 +1699,7 @@
         <v>0.5</v>
       </c>
       <c r="AQ6" t="n">
-        <v>0.03</v>
+        <v>0.038</v>
       </c>
     </row>
     <row r="7">
@@ -1969,7 +1969,7 @@
         <v>59</v>
       </c>
       <c r="B9" t="n">
-        <v>-0.000896673339502511</v>
+        <v>-0.00134262361139957</v>
       </c>
       <c r="C9" t="n">
         <v>1967.85312519324</v>
@@ -1990,10 +1990,10 @@
         <v>1189.81058417074</v>
       </c>
       <c r="I9" t="n">
-        <v>0.00314956198232288</v>
+        <v>0.00471596076438905</v>
       </c>
       <c r="J9" t="n">
-        <v>-351.24965174835</v>
+        <v>-351.249652124997</v>
       </c>
       <c r="K9" t="n">
         <v>-0.00431266486270832</v>
@@ -2002,7 +2002,7 @@
         <v>0.776152289421202</v>
       </c>
       <c r="M9" t="n">
-        <v>-0.000896994709920407</v>
+        <v>-0.00134310481173425</v>
       </c>
       <c r="N9" t="n">
         <v>1967.85309524445</v>
@@ -2023,10 +2023,10 @@
         <v>1191.88739650601</v>
       </c>
       <c r="T9" t="n">
-        <v>0.0122027456325354</v>
+        <v>0.0182716421983545</v>
       </c>
       <c r="U9" t="n">
-        <v>-1360.40329977177</v>
+        <v>-1360.40330127041</v>
       </c>
       <c r="V9" t="n">
         <v>-0.00431303955160245</v>
@@ -2041,13 +2041,13 @@
         <v>1965.1</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.0247478150697211</v>
+        <v>0.0370558590061263</v>
       </c>
       <c r="AA9" t="n">
         <v>7.07037944035506</v>
       </c>
       <c r="AB9" t="n">
-        <v>0.749045008064568</v>
+        <v>1.12157401087272</v>
       </c>
       <c r="AC9" t="n">
         <v>215</v>
@@ -2068,7 +2068,7 @@
         <v>54</v>
       </c>
       <c r="AI9" t="n">
-        <v>-0.000896994709920407</v>
+        <v>-0.00134310481173425</v>
       </c>
       <c r="AJ9" t="s">
         <v>49</v>
@@ -2092,7 +2092,7 @@
         <v>0.5</v>
       </c>
       <c r="AQ9" t="n">
-        <v>0.025</v>
+        <v>0.037</v>
       </c>
     </row>
     <row r="10">
@@ -2100,7 +2100,7 @@
         <v>60</v>
       </c>
       <c r="B10" t="n">
-        <v>-0.00184418313096271</v>
+        <v>-0.00276136660508839</v>
       </c>
       <c r="C10" t="n">
         <v>1959.48478975147</v>
@@ -2121,10 +2121,10 @@
         <v>1174.81938744492</v>
       </c>
       <c r="I10" t="n">
-        <v>0.00343515609905331</v>
+        <v>0.00514359218871097</v>
       </c>
       <c r="J10" t="n">
-        <v>-186.269792916936</v>
+        <v>-186.269804930386</v>
       </c>
       <c r="K10" t="n">
         <v>-0.00343379843307812</v>
@@ -2133,7 +2133,7 @@
         <v>0.591943829970496</v>
       </c>
       <c r="M10" t="n">
-        <v>-0.00185304295152627</v>
+        <v>-0.00277463275649197</v>
       </c>
       <c r="N10" t="n">
         <v>1959.48515153822</v>
@@ -2154,10 +2154,10 @@
         <v>1176.89852470093</v>
       </c>
       <c r="T10" t="n">
-        <v>0.0137876830019358</v>
+        <v>0.0206448314266356</v>
       </c>
       <c r="U10" t="n">
-        <v>-744.056309681297</v>
+        <v>-744.056357668656</v>
       </c>
       <c r="V10" t="n">
         <v>-0.00343443123213882</v>
@@ -2172,13 +2172,13 @@
         <v>1960.39</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.0256241133573898</v>
+        <v>0.0383679742657434</v>
       </c>
       <c r="AA10" t="n">
         <v>7.07037944035506</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.75019898291531</v>
+        <v>1.1233019019712</v>
       </c>
       <c r="AC10" t="n">
         <v>209</v>
@@ -2199,7 +2199,7 @@
         <v>54</v>
       </c>
       <c r="AI10" t="n">
-        <v>-0.00185304295152627</v>
+        <v>-0.00277463275649197</v>
       </c>
       <c r="AJ10" t="s">
         <v>49</v>
@@ -2223,7 +2223,7 @@
         <v>0.5</v>
       </c>
       <c r="AQ10" t="n">
-        <v>0.026</v>
+        <v>0.038</v>
       </c>
     </row>
     <row r="11">
@@ -2231,7 +2231,7 @@
         <v>61</v>
       </c>
       <c r="B11" t="n">
-        <v>-0.00912427231944504</v>
+        <v>-0.0136621252280381</v>
       </c>
       <c r="C11" t="n">
         <v>1960.00588042205</v>
@@ -2252,10 +2252,10 @@
         <v>992.699066812712</v>
       </c>
       <c r="I11" t="n">
-        <v>0.00406701760041921</v>
+        <v>0.00608969913486005</v>
       </c>
       <c r="J11" t="n">
-        <v>-44.5736104538643</v>
+        <v>-44.5735859774033</v>
       </c>
       <c r="K11" t="n">
         <v>0.0220353666416618</v>
@@ -2264,7 +2264,7 @@
         <v>0.0260987151539967</v>
       </c>
       <c r="M11" t="n">
-        <v>-0.00919506304382901</v>
+        <v>-0.0137681229128568</v>
       </c>
       <c r="N11" t="n">
         <v>1960.0085975169</v>
@@ -2285,10 +2285,10 @@
         <v>994.792146838149</v>
       </c>
       <c r="T11" t="n">
-        <v>0.0162751794377513</v>
+        <v>0.0243694411678126</v>
       </c>
       <c r="U11" t="n">
-        <v>-176.99910658768</v>
+        <v>-176.999009393329</v>
       </c>
       <c r="V11" t="n">
         <v>0.0220306303821657</v>
@@ -2303,13 +2303,13 @@
         <v>1958.02</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.0294663348681551</v>
+        <v>0.0441210808802915</v>
       </c>
       <c r="AA11" t="n">
         <v>7.07037944035506</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.74599588125286</v>
+        <v>1.11700843557211</v>
       </c>
       <c r="AC11" t="n">
         <v>180</v>
@@ -2330,7 +2330,7 @@
         <v>54</v>
       </c>
       <c r="AI11" t="n">
-        <v>-0.00919506304382901</v>
+        <v>-0.0137681229128568</v>
       </c>
       <c r="AJ11" t="s">
         <v>49</v>
@@ -2354,7 +2354,7 @@
         <v>0.5</v>
       </c>
       <c r="AQ11" t="n">
-        <v>0.029</v>
+        <v>0.044</v>
       </c>
     </row>
     <row r="12">
@@ -2624,7 +2624,7 @@
         <v>64</v>
       </c>
       <c r="B14" t="n">
-        <v>0.00232656221059133</v>
+        <v>0.00348365142545999</v>
       </c>
       <c r="C14" t="n">
         <v>1956.59973730689</v>
@@ -2645,10 +2645,10 @@
         <v>1078.76032223092</v>
       </c>
       <c r="I14" t="n">
-        <v>0.00314197576043525</v>
+        <v>0.00470459974720311</v>
       </c>
       <c r="J14" t="n">
-        <v>135.048001129386</v>
+        <v>135.047947473158</v>
       </c>
       <c r="K14" t="n">
         <v>-0.00225228831965074</v>
@@ -2657,7 +2657,7 @@
         <v>0.459878530173602</v>
       </c>
       <c r="M14" t="n">
-        <v>0.00248670441152616</v>
+        <v>0.00372343852593951</v>
       </c>
       <c r="N14" t="n">
         <v>1956.58787019111</v>
@@ -2678,10 +2678,10 @@
         <v>1080.81625267872</v>
       </c>
       <c r="T14" t="n">
-        <v>0.0129528271904879</v>
+        <v>0.0193947605494878</v>
       </c>
       <c r="U14" t="n">
-        <v>520.883267446263</v>
+        <v>520.883060492962</v>
       </c>
       <c r="V14" t="n">
         <v>-0.00212377449258661</v>
@@ -2696,13 +2696,13 @@
         <v>1953.64</v>
       </c>
       <c r="Z14" t="n">
-        <v>0.026309467166284</v>
+        <v>0.0393941809850092</v>
       </c>
       <c r="AA14" t="n">
         <v>7.07037944035506</v>
       </c>
       <c r="AB14" t="n">
-        <v>0.747937638288551</v>
+        <v>1.11991590335203</v>
       </c>
       <c r="AC14" t="n">
         <v>202</v>
@@ -2723,7 +2723,7 @@
         <v>54</v>
       </c>
       <c r="AI14" t="n">
-        <v>0.00248670441152616</v>
+        <v>0.00372343852593951</v>
       </c>
       <c r="AJ14" t="s">
         <v>49</v>
@@ -2747,7 +2747,7 @@
         <v>0.5</v>
       </c>
       <c r="AQ14" t="n">
-        <v>0.026</v>
+        <v>0.039</v>
       </c>
     </row>
     <row r="15">
@@ -2886,7 +2886,7 @@
         <v>66</v>
       </c>
       <c r="B16" t="n">
-        <v>0.00200375824116892</v>
+        <v>0.00375562601113106</v>
       </c>
       <c r="C16" t="n">
         <v>1955.11797165256</v>
@@ -2907,10 +2907,10 @@
         <v>1432.2008954568</v>
       </c>
       <c r="I16" t="n">
-        <v>0.00185008144977655</v>
+        <v>0.00346758916248442</v>
       </c>
       <c r="J16" t="n">
-        <v>92.3305722100128</v>
+        <v>92.3305236519037</v>
       </c>
       <c r="K16" t="n">
         <v>0.000631098192193646</v>
@@ -2919,7 +2919,7 @@
         <v>0.279735163285301</v>
       </c>
       <c r="M16" t="n">
-        <v>0.00213975894238031</v>
+        <v>0.00401053089960882</v>
       </c>
       <c r="N16" t="n">
         <v>1955.10628683101</v>
@@ -2940,10 +2940,10 @@
         <v>1434.22637386368</v>
       </c>
       <c r="T16" t="n">
-        <v>0.00767237573382132</v>
+        <v>0.0143802571223667</v>
       </c>
       <c r="U16" t="n">
-        <v>358.56262038968</v>
+        <v>358.562431815931</v>
       </c>
       <c r="V16" t="n">
         <v>0.00075504443126373</v>
@@ -2958,13 +2958,13 @@
         <v>1955.54</v>
       </c>
       <c r="Z16" t="n">
-        <v>0.0192623925470752</v>
+        <v>0.036103328735013</v>
       </c>
       <c r="AA16" t="n">
         <v>7.07037944035506</v>
       </c>
       <c r="AB16" t="n">
-        <v>0.746479818010103</v>
+        <v>1.39912039471771</v>
       </c>
       <c r="AC16" t="n">
         <v>275</v>
@@ -2985,7 +2985,7 @@
         <v>54</v>
       </c>
       <c r="AI16" t="n">
-        <v>0.00213975894238031</v>
+        <v>0.00401053089960882</v>
       </c>
       <c r="AJ16" t="s">
         <v>49</v>
@@ -3009,7 +3009,7 @@
         <v>0.5</v>
       </c>
       <c r="AQ16" t="n">
-        <v>0.019</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="17">

</xml_diff>